<commit_message>
feat: enrich Pertinence métier narrative paragraph with posture, resilience and peer comparability for T4 reports
</commit_message>
<xml_diff>
--- a/outputs/resultats/bnc/2025_t4_vs_2024_t4/comparison.xlsx
+++ b/outputs/resultats/bnc/2025_t4_vs_2024_t4/comparison.xlsx
@@ -597,7 +597,7 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-30T05:52:10.648561+00:00</t>
+          <t>2026-07-30T06:31:21.237102+00:00</t>
         </is>
       </c>
     </row>
@@ -1022,8 +1022,16 @@
         </is>
       </c>
       <c r="K10" s="3" t="inlineStr"/>
-      <c r="L10" s="3" t="inlineStr"/>
-      <c r="M10" s="3" t="inlineStr"/>
+      <c r="L10" s="3" t="inlineStr">
+        <is>
+          <t>Validé</t>
+        </is>
+      </c>
+      <c r="M10" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-30T06:31:21.935771+00:00</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">

</xml_diff>